<commit_message>
D->24 and D-> Done and sent for printing
</commit_message>
<xml_diff>
--- a/pre primary oral marks slip/lkg/lkg, marksleep.xlsx
+++ b/pre primary oral marks slip/lkg/lkg, marksleep.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\Third Term 2082\pre primary oral marks slip\lkg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E64FBD-97AC-4F14-8BE9-7905498F24E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0564B061-51FA-4BE8-B716-C2A4968BB85F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Roll</t>
   </si>
@@ -139,10 +139,13 @@
     <t>c</t>
   </si>
   <si>
-    <t>e</t>
-  </si>
-  <si>
     <t>a</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>LKG, Rhymes.</t>
   </si>
 </sst>
 </file>
@@ -168,7 +171,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -191,15 +194,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -516,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -524,92 +539,90 @@
     <col min="3" max="18" width="6.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="13.5" customHeight="1">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:18">
+      <c r="A1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+    </row>
+    <row r="2" spans="1:18" ht="13.5" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3">
+      <c r="C2" s="3">
         <v>1</v>
       </c>
-      <c r="D1" s="3">
+      <c r="D2" s="3">
         <v>2</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E2" s="3">
         <v>3</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F2" s="3">
         <v>4</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G2" s="3">
         <v>5</v>
       </c>
-      <c r="H1" s="3">
+      <c r="H2" s="3">
         <v>6</v>
       </c>
-      <c r="I1" s="3">
+      <c r="I2" s="3">
         <v>7</v>
       </c>
-      <c r="J1" s="3">
+      <c r="J2" s="3">
         <v>8</v>
       </c>
-      <c r="K1" s="3">
+      <c r="K2" s="3">
         <v>9</v>
       </c>
-      <c r="L1" s="3">
+      <c r="L2" s="3">
         <v>10</v>
       </c>
-      <c r="M1" s="3">
+      <c r="M2" s="3">
         <v>11</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N2" s="3">
+        <v>12</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="O1" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="13.5" customHeight="1">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
     </row>
     <row r="3" spans="1:18" ht="13.5" customHeight="1">
       <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -630,10 +643,10 @@
     </row>
     <row r="4" spans="1:18" ht="13.5" customHeight="1">
       <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -654,10 +667,10 @@
     </row>
     <row r="5" spans="1:18" ht="13.5" customHeight="1">
       <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -678,10 +691,10 @@
     </row>
     <row r="6" spans="1:18" ht="13.5" customHeight="1">
       <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -702,10 +715,10 @@
     </row>
     <row r="7" spans="1:18" ht="13.5" customHeight="1">
       <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -726,10 +739,10 @@
     </row>
     <row r="8" spans="1:18" ht="13.5" customHeight="1">
       <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -750,10 +763,10 @@
     </row>
     <row r="9" spans="1:18" ht="13.5" customHeight="1">
       <c r="A9" s="2">
+        <v>7</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -774,10 +787,10 @@
     </row>
     <row r="10" spans="1:18" ht="13.5" customHeight="1">
       <c r="A10" s="2">
+        <v>8</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -798,10 +811,10 @@
     </row>
     <row r="11" spans="1:18" ht="13.5" customHeight="1">
       <c r="A11" s="2">
+        <v>9</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -822,10 +835,10 @@
     </row>
     <row r="12" spans="1:18" ht="13.5" customHeight="1">
       <c r="A12" s="2">
+        <v>10</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -846,10 +859,10 @@
     </row>
     <row r="13" spans="1:18" ht="13.5" customHeight="1">
       <c r="A13" s="2">
+        <v>11</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -870,10 +883,10 @@
     </row>
     <row r="14" spans="1:18" ht="13.5" customHeight="1">
       <c r="A14" s="2">
+        <v>12</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -894,10 +907,10 @@
     </row>
     <row r="15" spans="1:18" ht="13.5" customHeight="1">
       <c r="A15" s="2">
+        <v>13</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -918,10 +931,10 @@
     </row>
     <row r="16" spans="1:18" ht="13.5" customHeight="1">
       <c r="A16" s="2">
+        <v>14</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -942,10 +955,10 @@
     </row>
     <row r="17" spans="1:18" ht="13.5" customHeight="1">
       <c r="A17" s="2">
+        <v>15</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -966,10 +979,10 @@
     </row>
     <row r="18" spans="1:18" ht="13.5" customHeight="1">
       <c r="A18" s="2">
+        <v>16</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -990,10 +1003,10 @@
     </row>
     <row r="19" spans="1:18" ht="13.5" customHeight="1">
       <c r="A19" s="2">
+        <v>17</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -1014,10 +1027,10 @@
     </row>
     <row r="20" spans="1:18" ht="13.5" customHeight="1">
       <c r="A20" s="2">
+        <v>18</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -1038,10 +1051,10 @@
     </row>
     <row r="21" spans="1:18" ht="13.5" customHeight="1">
       <c r="A21" s="2">
+        <v>19</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -1062,10 +1075,10 @@
     </row>
     <row r="22" spans="1:18" ht="13.5" customHeight="1">
       <c r="A22" s="2">
+        <v>20</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -1086,10 +1099,10 @@
     </row>
     <row r="23" spans="1:18" ht="13.5" customHeight="1">
       <c r="A23" s="2">
+        <v>21</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -1110,10 +1123,10 @@
     </row>
     <row r="24" spans="1:18" ht="13.5" customHeight="1">
       <c r="A24" s="2">
+        <v>22</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -1134,10 +1147,10 @@
     </row>
     <row r="25" spans="1:18" ht="13.5" customHeight="1">
       <c r="A25" s="2">
+        <v>23</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -1158,10 +1171,10 @@
     </row>
     <row r="26" spans="1:18" ht="13.5" customHeight="1">
       <c r="A26" s="2">
+        <v>24</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
@@ -1182,10 +1195,10 @@
     </row>
     <row r="27" spans="1:18" ht="13.5" customHeight="1">
       <c r="A27" s="2">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -1206,10 +1219,10 @@
     </row>
     <row r="28" spans="1:18" ht="13.5" customHeight="1">
       <c r="A28" s="2">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -1230,10 +1243,10 @@
     </row>
     <row r="29" spans="1:18" ht="13.5" customHeight="1">
       <c r="A29" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -1254,10 +1267,10 @@
     </row>
     <row r="30" spans="1:18" ht="13.5" customHeight="1">
       <c r="A30" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -1278,10 +1291,10 @@
     </row>
     <row r="31" spans="1:18" ht="13.5" customHeight="1">
       <c r="A31" s="2">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -1302,10 +1315,10 @@
     </row>
     <row r="32" spans="1:18" ht="13.5" customHeight="1">
       <c r="A32" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -1326,10 +1339,10 @@
     </row>
     <row r="33" spans="1:18" ht="13.5" customHeight="1">
       <c r="A33" s="2">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -1350,10 +1363,10 @@
     </row>
     <row r="34" spans="1:18" ht="13.5" customHeight="1">
       <c r="A34" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -1374,10 +1387,10 @@
     </row>
     <row r="35" spans="1:18" ht="13.5" customHeight="1">
       <c r="A35" s="2">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -1398,10 +1411,10 @@
     </row>
     <row r="36" spans="1:18" ht="13.5" customHeight="1">
       <c r="A36" s="2">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -1420,7 +1433,34 @@
       <c r="Q36" s="1"/>
       <c r="R36" s="1"/>
     </row>
+    <row r="37" spans="1:18" ht="13.5" customHeight="1">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
+      <c r="P37" s="1"/>
+      <c r="Q37" s="1"/>
+      <c r="R37" s="1"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:R1"/>
+  </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>